<commit_message>
Fix: email generation error, mobile sidebar nav, professional email template
- Fix session cookie overflow by stripping large summaries before session storage
- Fix mobile sidebar overlay stacking context (moved inside app-layout)
- Add auto-close sidebar on nav link click (mobile)
- Fix generate.html proj.readme -> proj.summary
- Fix github_project_agent return str -> return [] on error
- New professional email template: intro + 3 project dash-points + skills + signature
- Fixed signature block with full name, portfolio, GitHub, LinkedIn, phone
</commit_message>
<xml_diff>
--- a/1488e41a-a3c7-4bb4-9b57-0e093d4c6b12_job_application_tracker.xlsx
+++ b/1488e41a-a3c7-4bb4-9b57-0e093d4c6b12_job_application_tracker.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Recipient Email</t>
+          <t>Email Address</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -489,6 +489,28 @@
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>Sent</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-08 00:41:51</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AI &amp; Software Development Trainee (MTO)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>jobs@thedigitz.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Sent</t>
         </is>

</xml_diff>